<commit_message>
remove GDP in EUR from PCAF framework
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/pcaf/pcaf.xlsx
+++ b/dataland-framework-toolbox/inputs/pcaf/pcaf.xlsx
@@ -552,8 +552,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{88872740-29A9-40F2-B082-91B9EBCAB4F9}" name="pcaf" displayName="pcaf" ref="A1:O18" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:O18" xr:uid="{88872740-29A9-40F2-B082-91B9EBCAB4F9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{88872740-29A9-40F2-B082-91B9EBCAB4F9}" name="pcaf" displayName="pcaf" ref="A1:O17" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:O17" xr:uid="{88872740-29A9-40F2-B082-91B9EBCAB4F9}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{98390CE1-0D17-4424-91A3-E09917989074}" uniqueName="1" name="Field Identifier" queryTableFieldId="1"/>
     <tableColumn id="2" xr3:uid="{0CDDE416-A15D-4C75-B137-861C20BFFC57}" uniqueName="2" name="Category" queryTableFieldId="2" dataDxfId="13"/>
@@ -802,7 +802,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B1EF222-4BC7-4189-BBB6-74FE5797088E}">
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.54296875" bestFit="1" customWidth="1"/>
@@ -1047,7 +1047,7 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
         <v>37</v>
@@ -1056,13 +1056,13 @@
         <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="G6" t="s">
         <v>19</v>
@@ -1074,7 +1074,7 @@
         <v>42</v>
       </c>
       <c r="J6" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K6" t="s">
         <v>22</v>
@@ -1091,7 +1091,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
         <v>37</v>
@@ -1100,13 +1100,13 @@
         <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G7" t="s">
         <v>19</v>
@@ -1118,7 +1118,7 @@
         <v>42</v>
       </c>
       <c r="J7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="K7" t="s">
         <v>22</v>
@@ -1135,22 +1135,22 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
         <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G8" t="s">
         <v>19</v>
@@ -1179,7 +1179,7 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
         <v>37</v>
@@ -1188,13 +1188,13 @@
         <v>51</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G9" t="s">
         <v>19</v>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
         <v>37</v>
@@ -1232,13 +1232,13 @@
         <v>51</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G10" t="s">
         <v>19</v>
@@ -1247,7 +1247,7 @@
         <v>41</v>
       </c>
       <c r="I10" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J10" t="s">
         <v>43</v>
@@ -1267,22 +1267,22 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
         <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G11" t="s">
         <v>19</v>
@@ -1291,7 +1291,7 @@
         <v>41</v>
       </c>
       <c r="I11" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="J11" t="s">
         <v>43</v>
@@ -1311,7 +1311,7 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
         <v>37</v>
@@ -1320,13 +1320,13 @@
         <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="G12" t="s">
         <v>19</v>
@@ -1355,22 +1355,22 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F13" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="G13" t="s">
         <v>19</v>
@@ -1382,7 +1382,7 @@
         <v>42</v>
       </c>
       <c r="J13" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="K13" t="s">
         <v>22</v>
@@ -1399,7 +1399,7 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
         <v>68</v>
@@ -1408,13 +1408,13 @@
         <v>69</v>
       </c>
       <c r="D14" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E14" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G14" t="s">
         <v>19</v>
@@ -1423,7 +1423,7 @@
         <v>41</v>
       </c>
       <c r="I14" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J14" t="s">
         <v>73</v>
@@ -1443,7 +1443,7 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
         <v>68</v>
@@ -1452,13 +1452,13 @@
         <v>69</v>
       </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F15" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="G15" t="s">
         <v>19</v>
@@ -1467,7 +1467,7 @@
         <v>41</v>
       </c>
       <c r="I15" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="J15" t="s">
         <v>73</v>
@@ -1487,7 +1487,7 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
         <v>68</v>
@@ -1496,13 +1496,13 @@
         <v>69</v>
       </c>
       <c r="D16" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F16" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G16" t="s">
         <v>19</v>
@@ -1531,7 +1531,7 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
         <v>68</v>
@@ -1540,13 +1540,13 @@
         <v>69</v>
       </c>
       <c r="D17" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="E17" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G17" t="s">
         <v>19</v>
@@ -1570,50 +1570,6 @@
         <v>19</v>
       </c>
       <c r="N17" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="s">
-        <v>68</v>
-      </c>
-      <c r="C18" t="s">
-        <v>69</v>
-      </c>
-      <c r="D18" t="s">
-        <v>83</v>
-      </c>
-      <c r="E18" t="s">
-        <v>84</v>
-      </c>
-      <c r="F18" t="s">
-        <v>85</v>
-      </c>
-      <c r="G18" t="s">
-        <v>19</v>
-      </c>
-      <c r="H18" t="s">
-        <v>41</v>
-      </c>
-      <c r="I18" t="s">
-        <v>42</v>
-      </c>
-      <c r="J18" t="s">
-        <v>73</v>
-      </c>
-      <c r="K18" t="s">
-        <v>22</v>
-      </c>
-      <c r="L18" t="s">
-        <v>19</v>
-      </c>
-      <c r="M18" t="s">
-        <v>19</v>
-      </c>
-      <c r="N18" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>